<commit_message>
added message structure from the internet (common TC chargers)
</commit_message>
<xml_diff>
--- a/test/TestOBC/OBC_CAN_Matrix.xlsx
+++ b/test/TestOBC/OBC_CAN_Matrix.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marlin\Documents\tubcloud\clientsync\Projekte\Elektroauto\Code\eVCU\test\TestOBC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66F6C83-51EC-45EE-9B55-F6DF21ACE838}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C815873B-07B1-47D7-88C6-620A419A135F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{F4618D10-EC10-4C94-A047-6640BA6180C3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="4" xr2:uid="{F4618D10-EC10-4C94-A047-6640BA6180C3}"/>
   </bookViews>
   <sheets>
     <sheet name="BMS_OBC" sheetId="1" r:id="rId1"/>
     <sheet name="OBC_BMS_1" sheetId="2" r:id="rId2"/>
     <sheet name="OBC_BMS_2" sheetId="3" r:id="rId3"/>
     <sheet name="OBC_BMS_3" sheetId="4" r:id="rId4"/>
+    <sheet name="TC" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="157">
   <si>
     <t xml:space="preserve">Signal Name
 </t>
@@ -1529,6 +1530,27 @@
       </rPr>
       <t>220Ohm</t>
     </r>
+  </si>
+  <si>
+    <t>OBC_DCVoltage</t>
+  </si>
+  <si>
+    <t>DC output voltage</t>
+  </si>
+  <si>
+    <t>0.1V/bit offset: 0 from TC Charger CAN Matrix message 0x18FF50E5</t>
+  </si>
+  <si>
+    <t>OBC_DCCurrent</t>
+  </si>
+  <si>
+    <t>DC output current</t>
+  </si>
+  <si>
+    <t>0.1A/bit offset :0 from TC Charger CAN Matrix message 0x18FF50E5</t>
+  </si>
+  <si>
+    <t>from TC Charger CAN Matrix message 0x18FF50E5</t>
   </si>
 </sst>
 </file>
@@ -2073,7 +2095,7 @@
     <col min="16" max="16384" width="10.90625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="9" customFormat="1" ht="30">
+    <row r="1" spans="1:15" ht="30">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -2120,7 +2142,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="9" customFormat="1" ht="50">
+    <row r="2" spans="1:15" ht="50">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
@@ -2167,7 +2189,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:15" s="9" customFormat="1" ht="40">
+    <row r="3" spans="1:15" ht="40">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -2214,7 +2236,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:15" s="9" customFormat="1" ht="30">
+    <row r="4" spans="1:15" ht="30">
       <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
@@ -3865,4 +3887,353 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74032C26-4339-415B-95F0-F927AC473E98}">
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5"/>
+  <cols>
+    <col min="1" max="14" width="10.90625" style="9"/>
+    <col min="15" max="15" width="91.81640625" style="9" customWidth="1"/>
+    <col min="16" max="16384" width="10.90625" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="30">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="20">
+      <c r="A2" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="3">
+        <v>16</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="20">
+      <c r="A3" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" s="12" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="20">
+      <c r="A4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="30">
+      <c r="A5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="20">
+      <c r="A6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="20">
+      <c r="A7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O7" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F7" xr:uid="{7E082E39-E51D-47A4-9CC8-831ED3CBB276}">
+      <formula1>"Unsigned,Signed"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>